<commit_message>
chore: update Plaza Wise District dataset
</commit_message>
<xml_diff>
--- a/Plaza Wise District.xlsx
+++ b/Plaza Wise District.xlsx
@@ -5,17 +5,33 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Firefox Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\app\Map Core\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F785955-3DC8-4713-9C99-9CCE07223BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6AFB83-BE97-41C6-943F-D8507DA24D3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="S  N    Division    Area    Pla" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'S  N    Division    Area    Pla'!$A$1:$E$702</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -14702,6 +14718,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E702" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>